<commit_message>
docs: add Sprint 5 artifacts for React Native mobile migration
Add Sprint_Five_Artifacts.md with 7 requirements (IDs 30-36, 39 story
points) covering the MVP mobile app: Expo research spike, project setup,
map with geolocation, restaurant markers, detail modal, auth, and filters.
Update Requirements_Stack.xlsx with matching entries.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documentation/Requirements_Stack.xlsx
+++ b/documentation/Requirements_Stack.xlsx
@@ -335,7 +335,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="B2:F38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="8.710000000000001" customWidth="1" style="4" min="1" max="2"/>
@@ -863,7 +863,7 @@
       <c r="E28" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F28" t="n">
+      <c r="F28" s="0" t="n">
         <v>4</v>
       </c>
     </row>
@@ -882,7 +882,7 @@
       <c r="E29" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F29" t="n">
+      <c r="F29" s="0" t="n">
         <v>4</v>
       </c>
     </row>
@@ -901,7 +901,7 @@
       <c r="E30" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F30" s="0" t="n">
         <v>4</v>
       </c>
     </row>
@@ -924,23 +924,139 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" ht="14.25" customHeight="1" s="4"/>
-    <row r="33" ht="14.25" customHeight="1" s="4"/>
+    <row r="32" ht="14.25" customHeight="1" s="4">
+      <c r="B32" t="n">
+        <v>30</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Spike: Research React Native/Expo for mobile migration</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" ht="14.25" customHeight="1" s="4">
+      <c r="B33" t="n">
+        <v>31</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Initialize Expo React Native project</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5</v>
+      </c>
+    </row>
     <row r="34" ht="14.25" customHeight="1" s="4">
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-    </row>
-    <row r="35" ht="14.25" customHeight="1" s="4"/>
+      <c r="B34" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Display interactive map with user location (mobile)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25" customHeight="1" s="4">
+      <c r="B35" t="n">
+        <v>33</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Fetch and display nearby restaurants on map (mobile)</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>8</v>
+      </c>
+      <c r="E35" t="n">
+        <v>3</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5</v>
+      </c>
+    </row>
     <row r="36" ht="14.25" customHeight="1" s="4">
-      <c r="B36" s="3" t="n"/>
-      <c r="C36" s="3" t="n"/>
-      <c r="D36" s="3" t="n"/>
-      <c r="E36" s="3" t="n"/>
-    </row>
-    <row r="37" ht="14.25" customHeight="1" s="4"/>
-    <row r="38" ht="14.25" customHeight="1" s="4"/>
+      <c r="B36" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Restaurant detail modal (mobile)</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25" customHeight="1" s="4">
+      <c r="B37" t="n">
+        <v>35</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>User authentication — login and signup (mobile)</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25" customHeight="1" s="4">
+      <c r="B38" t="n">
+        <v>36</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Basic restaurant filters — cuisine, distance, price, rating (mobile)</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>5</v>
+      </c>
+      <c r="E38" t="n">
+        <v>5</v>
+      </c>
+      <c r="F38" t="n">
+        <v>5</v>
+      </c>
+    </row>
     <row r="39" ht="14.25" customHeight="1" s="4"/>
     <row r="40" ht="14.25" customHeight="1" s="4"/>
     <row r="41" ht="14.25" customHeight="1" s="4"/>

</xml_diff>